<commit_message>
Add Register to add and remove prod
</commit_message>
<xml_diff>
--- a/testdata/Playwright_Data.xlsx
+++ b/testdata/Playwright_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\om.korde\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F37EA3-27C0-4A23-95C4-BDFD9E7941AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{855F248D-34AD-43AD-AFEA-334C3440341E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24" yWindow="2436" windowWidth="23016" windowHeight="7584" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -46,9 +46,6 @@
     <t>Patil</t>
   </si>
   <si>
-    <t>amit1.patil1@testmail.com</t>
-  </si>
-  <si>
     <t>Test@1001</t>
   </si>
   <si>
@@ -107,16 +104,27 @@
   </si>
   <si>
     <t>FaxNumber</t>
+  </si>
+  <si>
+    <t>amit15.patil15@testmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -160,15 +168,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -506,34 +517,34 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -546,44 +557,47 @@
       <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{ABA22B27-B7E8-4B96-AEEF-0EAAB0515371}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>